<commit_message>
Show multiple daily items in cash flow template
</commit_message>
<xml_diff>
--- a/outputs/cash-flow-import-template/cash-flow-import-template.xlsx
+++ b/outputs/cash-flow-import-template/cash-flow-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="1" r:id="R2f4cad4abd784c95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rbafba1610bd84163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="1" r:id="Rfd6300a15b5f4d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R8db052e4e047416a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -406,92 +406,122 @@
         <x:v>Services</x:v>
       </x:c>
       <x:c r="C2" s="22" t="str">
-        <x:v>Hair service income</x:v>
+        <x:v>Haircut service</x:v>
       </x:c>
       <x:c r="D2" s="15" t="n">
-        <x:v>12000</x:v>
+        <x:v>3000</x:v>
       </x:c>
       <x:c r="E2" s="15" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F2" s="15" t="n">
         <x:f>D2-E2</x:f>
-        <x:v>12000</x:v>
+        <x:v>3000</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="n">
-        <x:v>46176.291666666664</x:v>
+        <x:v>46174.291666666664</x:v>
       </x:c>
       <x:c r="B3" s="17" t="str">
-        <x:v>Products &amp; Supplies</x:v>
+        <x:v>Services</x:v>
       </x:c>
       <x:c r="C3" s="23" t="str">
-        <x:v>Shampoo restock</x:v>
+        <x:v>Hair color service</x:v>
       </x:c>
       <x:c r="D3" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>9000</x:v>
       </x:c>
       <x:c r="E3" s="18" t="n">
-        <x:v>24500</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
         <x:f>D3-E3</x:f>
-        <x:v>-24500</x:v>
+        <x:v>9000</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="16" t="n">
-        <x:v>46178.291666666664</x:v>
+        <x:v>46174.291666666664</x:v>
       </x:c>
       <x:c r="B4" s="17" t="str">
-        <x:v>Utilities</x:v>
+        <x:v>POS Sales</x:v>
       </x:c>
       <x:c r="C4" s="23" t="str">
-        <x:v>Electricity bill</x:v>
+        <x:v>Shampoo product sale</x:v>
       </x:c>
       <x:c r="D4" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="E4" s="18" t="n">
-        <x:v>18000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="18" t="n">
         <x:f>D4-E4</x:f>
-        <x:v>-18000</x:v>
+        <x:v>2500</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="16"/>
-      <x:c r="B5" s="17"/>
-      <x:c r="C5" s="23"/>
-      <x:c r="D5" s="18"/>
-      <x:c r="E5" s="18"/>
+      <x:c r="A5" s="16" t="n">
+        <x:v>46174.291666666664</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>Products &amp; Supplies</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>Shampoo stock purchase</x:v>
+      </x:c>
+      <x:c r="D5" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="18" t="n">
+        <x:v>24500</x:v>
+      </x:c>
       <x:c r="F5" s="18" t="n">
         <x:f>D5-E5</x:f>
-        <x:v>0</x:v>
+        <x:v>-24500</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="16"/>
-      <x:c r="B6" s="17"/>
-      <x:c r="C6" s="23"/>
-      <x:c r="D6" s="18"/>
-      <x:c r="E6" s="18"/>
+      <x:c r="A6" s="16" t="n">
+        <x:v>46175.291666666664</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>Services</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="str">
+        <x:v>Facial service</x:v>
+      </x:c>
+      <x:c r="D6" s="18" t="n">
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="E6" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F6" s="18" t="n">
         <x:f>D6-E6</x:f>
-        <x:v>0</x:v>
+        <x:v>6000</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="16"/>
-      <x:c r="B7" s="17"/>
-      <x:c r="C7" s="23"/>
-      <x:c r="D7" s="18"/>
-      <x:c r="E7" s="18"/>
+      <x:c r="A7" s="16" t="n">
+        <x:v>46175.291666666664</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>Utilities</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str">
+        <x:v>Electricity bill</x:v>
+      </x:c>
+      <x:c r="D7" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="18" t="n">
+        <x:v>18000</x:v>
+      </x:c>
       <x:c r="F7" s="18" t="n">
         <x:f>D7-E7</x:f>
-        <x:v>0</x:v>
+        <x:v>-18000</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2713,22 +2743,22 @@
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="35" t="str">
-        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
+        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
-        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
+        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
       </x:c>
       <x:c r="C11" s="35" t="str">
-        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
+        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
       </x:c>
       <x:c r="D11" s="35" t="str">
-        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
+        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
       </x:c>
       <x:c r="E11" s="35" t="str">
-        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
+        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
       </x:c>
       <x:c r="F11" s="35" t="str">
-        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
+        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Revert "Show multiple daily items in cash flow template"
This reverts commit 49876c23883fe70b89409b10660ab3d36f62a7c6.
</commit_message>
<xml_diff>
--- a/outputs/cash-flow-import-template/cash-flow-import-template.xlsx
+++ b/outputs/cash-flow-import-template/cash-flow-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="1" r:id="Rfd6300a15b5f4d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R8db052e4e047416a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow" sheetId="1" r:id="R2f4cad4abd784c95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rbafba1610bd84163"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -406,122 +406,92 @@
         <x:v>Services</x:v>
       </x:c>
       <x:c r="C2" s="22" t="str">
-        <x:v>Haircut service</x:v>
+        <x:v>Hair service income</x:v>
       </x:c>
       <x:c r="D2" s="15" t="n">
-        <x:v>3000</x:v>
+        <x:v>12000</x:v>
       </x:c>
       <x:c r="E2" s="15" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F2" s="15" t="n">
         <x:f>D2-E2</x:f>
-        <x:v>3000</x:v>
+        <x:v>12000</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="n">
-        <x:v>46174.291666666664</x:v>
+        <x:v>46176.291666666664</x:v>
       </x:c>
       <x:c r="B3" s="17" t="str">
-        <x:v>Services</x:v>
+        <x:v>Products &amp; Supplies</x:v>
       </x:c>
       <x:c r="C3" s="23" t="str">
-        <x:v>Hair color service</x:v>
+        <x:v>Shampoo restock</x:v>
       </x:c>
       <x:c r="D3" s="18" t="n">
-        <x:v>9000</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E3" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>24500</x:v>
       </x:c>
       <x:c r="F3" s="18" t="n">
         <x:f>D3-E3</x:f>
-        <x:v>9000</x:v>
+        <x:v>-24500</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="16" t="n">
-        <x:v>46174.291666666664</x:v>
+        <x:v>46178.291666666664</x:v>
       </x:c>
       <x:c r="B4" s="17" t="str">
-        <x:v>POS Sales</x:v>
+        <x:v>Utilities</x:v>
       </x:c>
       <x:c r="C4" s="23" t="str">
-        <x:v>Shampoo product sale</x:v>
+        <x:v>Electricity bill</x:v>
       </x:c>
       <x:c r="D4" s="18" t="n">
-        <x:v>2500</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E4" s="18" t="n">
-        <x:v>0</x:v>
+        <x:v>18000</x:v>
       </x:c>
       <x:c r="F4" s="18" t="n">
         <x:f>D4-E4</x:f>
-        <x:v>2500</x:v>
+        <x:v>-18000</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="16" t="n">
-        <x:v>46174.291666666664</x:v>
-      </x:c>
-      <x:c r="B5" s="17" t="str">
-        <x:v>Products &amp; Supplies</x:v>
-      </x:c>
-      <x:c r="C5" s="23" t="str">
-        <x:v>Shampoo stock purchase</x:v>
-      </x:c>
-      <x:c r="D5" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="18" t="n">
-        <x:v>24500</x:v>
-      </x:c>
+      <x:c r="A5" s="16"/>
+      <x:c r="B5" s="17"/>
+      <x:c r="C5" s="23"/>
+      <x:c r="D5" s="18"/>
+      <x:c r="E5" s="18"/>
       <x:c r="F5" s="18" t="n">
         <x:f>D5-E5</x:f>
-        <x:v>-24500</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="16" t="n">
-        <x:v>46175.291666666664</x:v>
-      </x:c>
-      <x:c r="B6" s="17" t="str">
-        <x:v>Services</x:v>
-      </x:c>
-      <x:c r="C6" s="23" t="str">
-        <x:v>Facial service</x:v>
-      </x:c>
-      <x:c r="D6" s="18" t="n">
-        <x:v>6000</x:v>
-      </x:c>
-      <x:c r="E6" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="A6" s="16"/>
+      <x:c r="B6" s="17"/>
+      <x:c r="C6" s="23"/>
+      <x:c r="D6" s="18"/>
+      <x:c r="E6" s="18"/>
       <x:c r="F6" s="18" t="n">
         <x:f>D6-E6</x:f>
-        <x:v>6000</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="16" t="n">
-        <x:v>46175.291666666664</x:v>
-      </x:c>
-      <x:c r="B7" s="17" t="str">
-        <x:v>Utilities</x:v>
-      </x:c>
-      <x:c r="C7" s="23" t="str">
-        <x:v>Electricity bill</x:v>
-      </x:c>
-      <x:c r="D7" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="18" t="n">
-        <x:v>18000</x:v>
-      </x:c>
+      <x:c r="A7" s="16"/>
+      <x:c r="B7" s="17"/>
+      <x:c r="C7" s="23"/>
+      <x:c r="D7" s="18"/>
+      <x:c r="E7" s="18"/>
       <x:c r="F7" s="18" t="n">
         <x:f>D7-E7</x:f>
-        <x:v>-18000</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2743,22 +2713,22 @@
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="35" t="str">
-        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="B11" s="35" t="str">
-        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="C11" s="35" t="str">
-        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="D11" s="35" t="str">
-        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="E11" s="35" t="str">
-        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
       <x:c r="F11" s="35" t="str">
-        <x:v>Use one row per product, service, or expense. Repeat the same date on as many rows as needed for multiple items in one day. Delete the sample rows, add your own records, then upload from Cash Flow → Import.</x:v>
+        <x:v>Delete the sample rows on the Cash Flow sheet, add your own records, then upload the workbook from Cash Flow → Import. Keep the Closing formulas.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>